<commit_message>
docs(growth): prioritize measured conversion work
</commit_message>
<xml_diff>
--- a/outputs/project-tracker-2026-09-19/Comparador-Hardware-Project-Tracker.xlsx
+++ b/outputs/project-tracker-2026-09-19/Comparador-Hardware-Project-Tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R4d751181fcb64c67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R700f1cfe9c6248a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1109,7 +1109,7 @@
       <x:c r="R6" s="47"/>
       <x:c r="S6" s="35" t="n">
         <x:f>COUNTIF($E$10:$E$40,"In Progress")</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="T6" s="36"/>
       <x:c r="U6" s="36"/>
@@ -1123,7 +1123,7 @@
       <x:c r="Z6" s="40"/>
       <x:c r="AA6" s="38" t="n">
         <x:f>COUNTIF($F$10:$F$40,"P0")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="AB6" s="39"/>
       <x:c r="AC6" s="39"/>
@@ -1997,10 +1997,10 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="E17" s="8" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="F17" s="8" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="G17" s="49" t="n">
         <x:v>46287.5</x:v>
@@ -4105,7 +4105,7 @@
         <x:v>Not Started</x:v>
       </x:c>
       <x:c r="F40" s="15" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="G40" s="59" t="n">
         <x:v>46286.5</x:v>
@@ -4184,7 +4184,7 @@
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
       <x:c r="B41" s="53" t="str">
-        <x:v>Fuentes: REVISION-Y-PLAN.md; BACKLOG.csv; METRICAS.csv; VALIDACION.md; Search Console y GA4 consultados el 21/09/2026. GSC 23/08–19/09 vs 26/07–22/08: 296 vs 192 clics, 14 mil vs 9,55 mil impresiones, CTR 2,1% vs 2,0%, posición 8,4 vs 8,5. Auditoría GSC: 3.187 indexadas / 326 no indexadas; sitemap correcto con 29 páginas descubiertas; HTTPS 31/0; 2 enlaces externos y 7.751 internos; 662 oportunidades Merchant; sin acciones manuales ni problemas de seguridad; sin datos CrUX. La prueba en vivo de la guía de 2 millones fue disponible e indexable, pero la validación 5xx sigue iniciada. GA4 24/08–20/09: 143 usuarios, 512 eventos, 178 page_view y 18 click; generate_lead aún no aparece. Las fechas futuras son planificación y se revisan semanalmente.</x:v>
+        <x:v>Fuentes: REVISION-Y-PLAN.md; BACKLOG.csv; METRICAS.csv; VALIDACION.md; Search Console y GA4 consultados el 21/09/2026. GSC 23/08–19/09 vs 26/07–22/08: 296 vs 192 clics, 14 mil vs 9,55 mil impresiones, CTR 2,1% vs 2,0%, posición 8,4 vs 8,5. Auditoría GSC: 3.187 indexadas / 326 no indexadas; sitemap correcto con 29 páginas descubiertas; HTTPS 31/0; 2 enlaces externos y 7.751 internos; 662 oportunidades Merchant; sin acciones manuales ni problemas de seguridad; sin datos CrUX. GA4 24/08–20/09: 143 usuarios, 512 eventos, 178 page_view y 18 click; generate_lead aún no aparece. Jev 21/09: embudo/CTA 64% (confianza 0,56); enlaces/rich results 39% y asociación GA4 32% como segundo orden (confianza 0,23); Merchant 6% y outreach 26% a favor. G07 pasa a P0/en curso; G17 a P1. Las fechas futuras son planificación y se revisan semanalmente.</x:v>
       </x:c>
       <x:c r="C41" s="54"/>
       <x:c r="D41" s="54"/>

</xml_diff>